<commit_message>
Run DangKy suite with 10 data rows in CI
</commit_message>
<xml_diff>
--- a/Tour_booking_Chip3chip_system/Data Files/Data_DangKy.xlsx
+++ b/Tour_booking_Chip3chip_system/Data Files/Data_DangKy.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_DangKy" sheetId="1" r:id="R3e121ffb7aa3484a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_DangKy" sheetId="1" r:id="Rcf9225b8b9114f60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -246,8 +246,8 @@
     <x:col min="1" max="1" width="10.880000114440918" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="9.130000114440918" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="8.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="15.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12.75" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16.75" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15.75" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="10.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="13.880000114440918" hidden="0" customWidth="1"/>
   </x:cols>
@@ -344,6 +344,167 @@
         <x:v>Password123</x:v>
       </x:c>
     </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>Pham Thi D</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>1995-02-28</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>0904445566</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>test4@example.com</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>Quan 7, TP HCM</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>Password123</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>Password123</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>Hoang Van E</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>2001-12-31</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>0905556677</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>test5@example.com</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>Thu Duc, TP HCM</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>Password123</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>Password123</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>Do Thi F</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>1990-05-05</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>0906667788</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>test6@example.com</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>Binh Thanh, TP HCM</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>Password123</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>Password123</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>Bui Van G</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>1999-01-01</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>0907778899</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>test7@example.com</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>Tan Binh, TP HCM</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>Password123</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>Password123</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>Vo Thi H</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>1999-02-02</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>0908889900</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>test8@example.com</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>Go Vap, TP HCM</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>Password123</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>Password123</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>Dang Van I</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>1999-03-03</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>0910001122</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>test9@example.com</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>Phu Nhuan, TP HCM</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>Password123</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>Password123</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>Mai Thi K</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>1999-04-04</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>0911112233</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>test10@example.com</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>Quan 10, TP HCM</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>Password123</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>Password123</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>